<commit_message>
Protect shared Workday runtime bindings across targets
Reject conflicting connection selections for co-located tracked targets before Runtime mutations, while preserving identical-binding reuse and independent environments. Align the Workday workbook certificate recovery with the completed Entra handoff.

Copilot-Session: 8534f8ab-983a-4aea-8732-3ebce2dde3c1
</commit_message>
<xml_diff>
--- a/solutions/ess-maker-skills/src/skills/connect/workday/assets/workday-admin-workbook.xlsx
+++ b/solutions/ess-maker-skills/src/skills/connect/workday/assets/workday-admin-workbook.xlsx
@@ -136,8 +136,8 @@
 3. Find 'Certificate expiration date' (and 'Certificate thumbprint') on the Microsoft Entra worksheet or the agent handoff.</t>
   </si>
   <si>
-    <t>The public key's expiration date must exactly match the 'Certificate expiration date' on the Microsoft Entra worksheet.
-If the dates differ, the wrong certificate was uploaded - get the active certificate from the Microsoft Entra admin and repeat the Certificate row.</t>
+    <t>Exactly match the public key's expiration date to 'Certificate expiration date' on the Entra worksheet.
+For mismatches, correct Workday using the certificate already transferred during the completed Entra handoff. Re-engage Entra only for independently verified certificate drift.</t>
   </si>
   <si>
     <t>1. Run the View API Client task.

</xml_diff>

<commit_message>
Fix Workday discovery and workbook guidance
Copilot-Session: 8534f8ab-983a-4aea-8732-3ebce2dde3c1
</commit_message>
<xml_diff>
--- a/solutions/ess-maker-skills/src/skills/connect/workday/assets/workday-admin-workbook.xlsx
+++ b/solutions/ess-maker-skills/src/skills/connect/workday/assets/workday-admin-workbook.xlsx
@@ -140,9 +140,9 @@
 For mismatches, correct Workday using the certificate already transferred during the completed Entra handoff. Re-engage Entra only for independently verified certificate drift.</t>
   </si>
   <si>
-    <t>1. Run the View API Client task.
-2. Select the approved signed-in employee API client (Client Grant Type = SAML Bearer) that you reused or registered.
-3. Locate the Client ID field.</t>
+    <t>1. Complete row 11 (API client access) first: reuse an approved client or register one if none exists.
+2. Return here and to rows 6-8 to capture the client ID and endpoints.
+3. Run View API Client, select the client verified in row 11, and locate Client ID.</t>
   </si>
   <si>
     <t>Copy the Client ID exactly as shown. The client ID isn't a secret.
@@ -203,7 +203,7 @@
 - Limited or test population - the intended Workday security group and test employee access are configured</t>
   </si>
   <si>
-    <t>1. Run the View API Client task and open the signed-in employee API client.
+    <t>1. Check for an approved signed-in employee API client. If none exists, go to step 3 and register one. Otherwise, run View API Client and open it.
 2. Check Client Grant Type, Include Workday Owned Scope, and Scope (Functional Areas).
 3. Reuse an existing approved client only if all settings match. Otherwise run the Register API Client task with:
    - Client Grant Type: SAML Bearer
@@ -693,7 +693,7 @@
       </c>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" ht="100" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>

</xml_diff>